<commit_message>
feat: add accounting and logistics prompts, update README and sample data for new use cases
</commit_message>
<xml_diff>
--- a/sample-data/factory_issues_sample.xlsx
+++ b/sample-data/factory_issues_sample.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE64EDCA-577F-4260-ACD0-3099197FA3E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="factory_issues" sheetId="1" r:id="rId1"/>
@@ -444,13 +444,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="98.42578125" customWidth="1"/>
+    <col min="2" max="2" width="98.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -458,7 +458,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -466,7 +466,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -474,7 +474,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -482,7 +482,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -490,7 +490,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -498,7 +498,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
@@ -506,7 +506,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
@@ -514,7 +514,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -522,7 +522,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
@@ -530,7 +530,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>

</xml_diff>